<commit_message>
Add functionality to the website.
</commit_message>
<xml_diff>
--- a/mau_import_san_pham.xlsx
+++ b/mau_import_san_pham.xlsx
@@ -1,21 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\Desktop\font_end\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F6EA65B-B32D-48ED-A289-271CBD0DF52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8482A4A-CDDE-423B-BD76-467559C107CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -70,12 +81,6 @@
     <t>variant_quantities</t>
   </si>
   <si>
-    <t>Áo thun basic</t>
-  </si>
-  <si>
-    <t>Áo thun cotton co giãn</t>
-  </si>
-  <si>
     <t>[{"color":"Đen","size":"M","quantity":10},{"color":"Trắng","size":"L","quantity":8}]</t>
   </si>
   <si>
@@ -110,6 +115,22 @@
   </si>
   <si>
     <t>ao-thun-nam</t>
+  </si>
+  <si>
+    <t>Áo thun nam phối tay Exdry Peformance World Cup</t>
+  </si>
+  <si>
+    <t>- Công nghệ: Ex-Dry
+- Mã sản phẩm: DFKGH454
+- Chất liệu: 100% Rec. Polyester
+Vải tái chế thân thiện môi trường
+- Kiểu dáng: Regular fit
+Mẫu cao 1m8, nặng 70kg - Size XL
+Phù hợp
+Mặc hàng ngày và các hoạt động thể thao
+- Tính năng: Thoáng khí và co giãn
+- Bảo quản: Giặt máy nhẹ - Ủi ở nhiệt độ thấp
+Không giặt khô - Không dùng chất tẩy.'</t>
   </si>
 </sst>
 </file>
@@ -154,12 +175,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -536,52 +560,52 @@
     </row>
     <row r="2" spans="1:16" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1">
-        <v>199000</v>
+        <v>399000</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="G2" s="1">
         <v>10</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="M2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>